<commit_message>
Remove standalone figure titles and enforce caption-only descriptions
</commit_message>
<xml_diff>
--- a/plot_data/fig1.xlsx
+++ b/plot_data/fig1.xlsx
@@ -2554,7 +2554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2607,13 +2607,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>question</t>
+          <t>data_heading</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>How do model structure and input information
-jointly influence phenology transferability?</t>
+          <t>Data and provenance</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -2626,78 +2625,82 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>center</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>qualified_data</t>
+        </is>
+      </c>
       <c r="G2" t="b">
         <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>9.5</v>
+        <v>0.8</v>
       </c>
       <c r="I2" t="n">
-        <v>18.25</v>
+        <v>16.73</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>data_heading</t>
+          <t>data_body</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
-        <is>
-          <t>Data and provenance</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>12</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>bold</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>left</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>qualified_data</t>
-        </is>
-      </c>
-      <c r="G3" t="b">
-        <v>1</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="I3" t="n">
-        <v>16.73</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>data_body</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
         <is>
           <t>Observed maize event dates
 Daily weather at native cells
 Seven BBCH endpoints</t>
         </is>
       </c>
+      <c r="C3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>qualified_data</t>
+        </is>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I3" t="n">
+        <v>15.55</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>control_heading</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Calibration and testing</t>
+        </is>
+      </c>
       <c r="C4" t="n">
         <v>12</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>bold</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -2707,77 +2710,77 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>qualified_data</t>
+          <t>separation</t>
         </is>
       </c>
       <c r="G4" t="b">
         <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>0.8</v>
+        <v>10.3</v>
       </c>
       <c r="I4" t="n">
-        <v>15.55</v>
+        <v>16.73</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>control_heading</t>
+          <t>control_body</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
-        <is>
-          <t>Calibration and testing</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>12</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>bold</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>left</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>separation</t>
-        </is>
-      </c>
-      <c r="G5" t="b">
-        <v>1</v>
-      </c>
-      <c r="H5" t="n">
-        <v>10.3</v>
-      </c>
-      <c r="I5" t="n">
-        <v>16.73</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>control_body</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
         <is>
           <t>Fitting data end by 2010
 5 folds · 50-km spatial blocks
 25-km cell-centre buffer</t>
         </is>
       </c>
+      <c r="C5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>separation</t>
+        </is>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="I5" t="n">
+        <v>15.55</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>models_heading</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Six model formulations</t>
+        </is>
+      </c>
       <c r="C6" t="n">
         <v>12</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>bold</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -2787,28 +2790,28 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>separation</t>
+          <t>models</t>
         </is>
       </c>
       <c r="G6" t="b">
         <v>1</v>
       </c>
       <c r="H6" t="n">
-        <v>10.3</v>
+        <v>0.8</v>
       </c>
       <c r="I6" t="n">
-        <v>15.55</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>models_heading</t>
+          <t>model_T</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Six model formulations</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -2816,38 +2819,39 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>bold</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>center</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>models</t>
+          <t>T</t>
         </is>
       </c>
       <c r="G7" t="b">
         <v>1</v>
       </c>
       <c r="H7" t="n">
-        <v>0.8</v>
+        <v>2.06</v>
       </c>
       <c r="I7" t="n">
-        <v>13.5</v>
+        <v>12.37</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>model_T</t>
+          <t>model_nonlinear_T</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>Nonlinear
+T</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -2865,14 +2869,14 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>nonlinear_T</t>
         </is>
       </c>
       <c r="G8" t="b">
         <v>1</v>
       </c>
       <c r="H8" t="n">
-        <v>2.06</v>
+        <v>5.03</v>
       </c>
       <c r="I8" t="n">
         <v>12.37</v>
@@ -2881,13 +2885,13 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>model_nonlinear_T</t>
+          <t>model_residual_RF</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Nonlinear
-T</t>
+          <t>Residual
+RF</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -2905,14 +2909,14 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>nonlinear_T</t>
+          <t>residual_RF</t>
         </is>
       </c>
       <c r="G9" t="b">
         <v>1</v>
       </c>
       <c r="H9" t="n">
-        <v>5.03</v>
+        <v>8</v>
       </c>
       <c r="I9" t="n">
         <v>12.37</v>
@@ -2921,13 +2925,13 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>model_residual_RF</t>
+          <t>model_residual_MLP</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
           <t>Residual
-RF</t>
+MLP</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -2945,14 +2949,14 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>residual_RF</t>
+          <t>residual_MLP</t>
         </is>
       </c>
       <c r="G10" t="b">
         <v>1</v>
       </c>
       <c r="H10" t="n">
-        <v>8</v>
+        <v>10.97</v>
       </c>
       <c r="I10" t="n">
         <v>12.37</v>
@@ -2961,13 +2965,13 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>model_residual_MLP</t>
+          <t>model_thermal_transformer</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Residual
-MLP</t>
+          <t>Thermal
+Transformer</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -2985,14 +2989,14 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>residual_MLP</t>
+          <t>thermal_transformer</t>
         </is>
       </c>
       <c r="G11" t="b">
         <v>1</v>
       </c>
       <c r="H11" t="n">
-        <v>10.97</v>
+        <v>13.94</v>
       </c>
       <c r="I11" t="n">
         <v>12.37</v>
@@ -3001,13 +3005,13 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>model_thermal_transformer</t>
+          <t>model_support_blend</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Thermal
-Transformer</t>
+          <t>Support
+blend</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -3025,14 +3029,14 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>thermal_transformer</t>
+          <t>support_blend</t>
         </is>
       </c>
       <c r="G12" t="b">
         <v>1</v>
       </c>
       <c r="H12" t="n">
-        <v>13.94</v>
+        <v>16.91</v>
       </c>
       <c r="I12" t="n">
         <v>12.37</v>
@@ -3041,13 +3045,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>model_support_blend</t>
+          <t>benchmark_panel</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Support
-blend</t>
+          <t>(a)</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -3055,38 +3058,38 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>bold</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>left</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>support_blend</t>
+          <t>benchmark</t>
         </is>
       </c>
       <c r="G13" t="b">
         <v>1</v>
       </c>
       <c r="H13" t="n">
-        <v>16.91</v>
+        <v>0.8</v>
       </c>
       <c r="I13" t="n">
-        <v>12.37</v>
+        <v>10.12</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>benchmark_panel</t>
+          <t>benchmark_heading</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>(a)</t>
+          <t>Model performance</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -3111,7 +3114,7 @@
         <v>1</v>
       </c>
       <c r="H14" t="n">
-        <v>0.8</v>
+        <v>1.55</v>
       </c>
       <c r="I14" t="n">
         <v>10.12</v>
@@ -3120,61 +3123,61 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>benchmark_heading</t>
+          <t>benchmark_body</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
-        <is>
-          <t>Model performance</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>12</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>bold</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>left</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>benchmark</t>
-        </is>
-      </c>
-      <c r="G15" t="b">
-        <v>1</v>
-      </c>
-      <c r="H15" t="n">
-        <v>1.55</v>
-      </c>
-      <c r="I15" t="n">
-        <v>10.12</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>benchmark_body</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
         <is>
           <t>80 sites × 8 years · 3 draws
 Random / coverage sampling
 Stage errors; benefit and harm</t>
         </is>
       </c>
+      <c r="C15" t="n">
+        <v>12</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>benchmark</t>
+        </is>
+      </c>
+      <c r="G15" t="b">
+        <v>1</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I15" t="n">
+        <v>8.869999999999999</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>local_panel</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>(b)</t>
+        </is>
+      </c>
       <c r="C16" t="n">
         <v>12</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>bold</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -3184,28 +3187,28 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>benchmark</t>
+          <t>local</t>
         </is>
       </c>
       <c r="G16" t="b">
         <v>1</v>
       </c>
       <c r="H16" t="n">
-        <v>0.8</v>
+        <v>10.3</v>
       </c>
       <c r="I16" t="n">
-        <v>8.869999999999999</v>
+        <v>10.12</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>local_panel</t>
+          <t>local_heading</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>(b)</t>
+          <t>Local information</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -3230,7 +3233,7 @@
         <v>1</v>
       </c>
       <c r="H17" t="n">
-        <v>10.3</v>
+        <v>11.05</v>
       </c>
       <c r="I17" t="n">
         <v>10.12</v>
@@ -3239,61 +3242,61 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>local_heading</t>
+          <t>local_body</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
-        <is>
-          <t>Local information</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>12</v>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>bold</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>left</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>local</t>
-        </is>
-      </c>
-      <c r="G18" t="b">
-        <v>1</v>
-      </c>
-      <c r="H18" t="n">
-        <v>11.05</v>
-      </c>
-      <c r="I18" t="n">
-        <v>10.12</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>local_body</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
         <is>
           <t>0, 1, 3 or 5 past local years
 80-site coverage fit · 1 draw
 Five models; shared date offsets</t>
         </is>
       </c>
+      <c r="C18" t="n">
+        <v>12</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="G18" t="b">
+        <v>1</v>
+      </c>
+      <c r="H18" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="I18" t="n">
+        <v>8.869999999999999</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>transfer_panel</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>(c)</t>
+        </is>
+      </c>
       <c r="C19" t="n">
         <v>12</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>bold</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -3303,28 +3306,28 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>local</t>
+          <t>transfer</t>
         </is>
       </c>
       <c r="G19" t="b">
         <v>1</v>
       </c>
       <c r="H19" t="n">
-        <v>10.3</v>
+        <v>0.8</v>
       </c>
       <c r="I19" t="n">
-        <v>8.869999999999999</v>
+        <v>6.27</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>transfer_panel</t>
+          <t>transfer_heading</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>(c)</t>
+          <t>Environmental transfer</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -3349,7 +3352,7 @@
         <v>1</v>
       </c>
       <c r="H20" t="n">
-        <v>0.8</v>
+        <v>1.55</v>
       </c>
       <c r="I20" t="n">
         <v>6.27</v>
@@ -3358,61 +3361,61 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>transfer_heading</t>
+          <t>transfer_body</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
-        <is>
-          <t>Environmental transfer</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>12</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>bold</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>left</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>transfer</t>
-        </is>
-      </c>
-      <c r="G21" t="b">
-        <v>1</v>
-      </c>
-      <c r="H21" t="n">
-        <v>1.55</v>
-      </c>
-      <c r="I21" t="n">
-        <v>6.27</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>transfer_body</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
         <is>
           <t>40 sites × 8 years · 3 draws
 5 temperature zones + pooled
 Paired transfer loss and distance</t>
         </is>
       </c>
+      <c r="C21" t="n">
+        <v>12</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>transfer</t>
+        </is>
+      </c>
+      <c r="G21" t="b">
+        <v>1</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I21" t="n">
+        <v>5.02</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>weather_panel</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>(d)</t>
+        </is>
+      </c>
       <c r="C22" t="n">
         <v>12</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>bold</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -3422,28 +3425,28 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>transfer</t>
+          <t>weather</t>
         </is>
       </c>
       <c r="G22" t="b">
         <v>1</v>
       </c>
       <c r="H22" t="n">
-        <v>0.8</v>
+        <v>10.3</v>
       </c>
       <c r="I22" t="n">
-        <v>5.02</v>
+        <v>6.27</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>weather_panel</t>
+          <t>weather_heading</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>(d)</t>
+          <t>Weather inputs</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3468,7 +3471,7 @@
         <v>1</v>
       </c>
       <c r="H23" t="n">
-        <v>10.3</v>
+        <v>11.05</v>
       </c>
       <c r="I23" t="n">
         <v>6.27</v>
@@ -3477,61 +3480,61 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>weather_heading</t>
+          <t>weather_body</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
-        <is>
-          <t>Weather inputs</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>12</v>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>bold</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>left</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>weather</t>
-        </is>
-      </c>
-      <c r="G24" t="b">
-        <v>1</v>
-      </c>
-      <c r="H24" t="n">
-        <v>11.05</v>
-      </c>
-      <c r="I24" t="n">
-        <v>6.27</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>weather_body</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
         <is>
           <t>40 sites × 4 years · 3 draws
 DWD station / ERA5-Land inputs
 Weather swaps and refitting</t>
         </is>
       </c>
+      <c r="C24" t="n">
+        <v>12</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
+      <c r="G24" t="b">
+        <v>1</v>
+      </c>
+      <c r="H24" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="I24" t="n">
+        <v>5.02</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>evaluation_heading</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Paired evaluation under specified conditions</t>
+        </is>
+      </c>
       <c r="C25" t="n">
         <v>12</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>bold</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -3541,96 +3544,57 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>weather</t>
+          <t>evaluation</t>
         </is>
       </c>
       <c r="G25" t="b">
         <v>1</v>
       </c>
       <c r="H25" t="n">
-        <v>10.3</v>
+        <v>0.8</v>
       </c>
       <c r="I25" t="n">
-        <v>5.02</v>
+        <v>2.53</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>evaluation_heading</t>
+          <t>evaluation_body</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
-        <is>
-          <t>Paired evaluation under specified conditions</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>12</v>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>bold</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>left</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>evaluation</t>
-        </is>
-      </c>
-      <c r="G26" t="b">
-        <v>1</v>
-      </c>
-      <c r="H26" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="I26" t="n">
-        <v>2.53</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>evaluation_body</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
         <is>
           <t>2011–2025 outcomes; weather cohort: 2011–2024
 Penalised MAE; equal endpoint weights · Invalid dates: 366 d
 95% conditional intervals · Spatial / station groups</t>
         </is>
       </c>
-      <c r="C27" t="n">
+      <c r="C26" t="n">
         <v>12</v>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>left</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>evaluation</t>
         </is>
       </c>
-      <c r="G27" t="b">
+      <c r="G26" t="b">
         <v>1</v>
       </c>
-      <c r="H27" t="n">
+      <c r="H26" t="n">
         <v>0.8</v>
       </c>
-      <c r="I27" t="n">
+      <c r="I26" t="n">
         <v>1.4</v>
       </c>
     </row>

</xml_diff>